<commit_message>
fix and update upload Excel
</commit_message>
<xml_diff>
--- a/backend/nodejs/templates/KPM_Import_Product.xlsx
+++ b/backend/nodejs/templates/KPM_Import_Product.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TP\Desktop\KPM\backend\nodejs\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8FFA737-FFCF-43E4-A3ED-1F03DDC3D091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{407A64FB-F31E-430C-AD2F-F914B0A5A0EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EBB0906C-0CA5-40FD-8E8B-61911B6F40BC}"/>
   </bookViews>
@@ -648,6 +648,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -684,6 +685,15 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -702,16 +712,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1130,35 +1130,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
-      <c r="A1" s="17" t="e" vm="1">
+      <c r="A1" s="18" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="23"/>
     </row>
     <row r="2" spans="1:19" ht="31.8" thickBot="1">
-      <c r="A2" s="18"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="25"/>
+      <c r="A2" s="19"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="26"/>
       <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:19" ht="28.8" customHeight="1" thickBot="1">
-      <c r="A3" s="19"/>
-      <c r="B3" s="26" t="s">
+      <c r="A3" s="20"/>
+      <c r="B3" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="29"/>
     </row>
     <row r="4" spans="1:19" ht="23.4">
       <c r="A4" s="14" t="s">
@@ -1187,9 +1187,9 @@
       <c r="S4" s="2"/>
     </row>
     <row r="5" spans="1:19" ht="16.8">
-      <c r="A5" s="38"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
       <c r="D5" s="15"/>
       <c r="E5" s="15"/>
       <c r="F5" s="15"/>
@@ -1201,9 +1201,9 @@
       <c r="S5" s="3"/>
     </row>
     <row r="6" spans="1:19" ht="16.8">
-      <c r="A6" s="38"/>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
@@ -1215,9 +1215,9 @@
       <c r="S6" s="3"/>
     </row>
     <row r="7" spans="1:19" ht="16.8">
-      <c r="A7" s="38"/>
-      <c r="B7" s="38"/>
-      <c r="C7" s="38"/>
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
@@ -1226,9 +1226,9 @@
       <c r="Q7" s="3"/>
     </row>
     <row r="8" spans="1:19" ht="18">
-      <c r="A8" s="38"/>
-      <c r="B8" s="38"/>
-      <c r="C8" s="38"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
@@ -1238,9 +1238,9 @@
       <c r="S8" s="4"/>
     </row>
     <row r="9" spans="1:19" ht="18">
-      <c r="A9" s="38"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
@@ -1251,9 +1251,9 @@
       <c r="S9" s="3"/>
     </row>
     <row r="10" spans="1:19" ht="18">
-      <c r="A10" s="38"/>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -1265,9 +1265,9 @@
       <c r="S10" s="3"/>
     </row>
     <row r="11" spans="1:19" ht="16.8">
-      <c r="A11" s="38"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38"/>
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
@@ -1956,10 +1956,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="33.6">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="33" t="s">
         <v>37</v>
       </c>
       <c r="C2" s="9" t="s">
@@ -1970,14 +1970,14 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="16.8">
-      <c r="A3" s="36"/>
-      <c r="B3" s="30"/>
+      <c r="A3" s="31"/>
+      <c r="B3" s="34"/>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
     </row>
     <row r="4" spans="1:4" ht="16.8">
-      <c r="A4" s="36"/>
-      <c r="B4" s="30"/>
+      <c r="A4" s="31"/>
+      <c r="B4" s="34"/>
       <c r="C4" s="10" t="s">
         <v>39</v>
       </c>
@@ -1986,52 +1986,52 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="16.8">
-      <c r="A5" s="36"/>
-      <c r="B5" s="30"/>
+      <c r="A5" s="31"/>
+      <c r="B5" s="34"/>
       <c r="C5" s="11"/>
       <c r="D5" s="11"/>
     </row>
     <row r="6" spans="1:4" ht="34.200000000000003" thickBot="1">
-      <c r="A6" s="37"/>
-      <c r="B6" s="31"/>
+      <c r="A6" s="32"/>
+      <c r="B6" s="35"/>
       <c r="C6" s="12" t="s">
         <v>40</v>
       </c>
       <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:4" ht="16.8">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="33" t="s">
         <v>37</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="33" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16.8">
-      <c r="A8" s="36"/>
-      <c r="B8" s="30"/>
+      <c r="A8" s="31"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="30"/>
+      <c r="D8" s="34"/>
     </row>
     <row r="9" spans="1:4" ht="34.200000000000003" thickBot="1">
-      <c r="A9" s="37"/>
-      <c r="B9" s="31"/>
+      <c r="A9" s="32"/>
+      <c r="B9" s="35"/>
       <c r="C9" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="31"/>
+      <c r="D9" s="35"/>
     </row>
     <row r="10" spans="1:4" ht="16.8">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="33" t="s">
         <v>37</v>
       </c>
       <c r="C10" s="9" t="s">
@@ -2042,14 +2042,14 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="16.8">
-      <c r="A11" s="36"/>
-      <c r="B11" s="30"/>
+      <c r="A11" s="31"/>
+      <c r="B11" s="34"/>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
     </row>
     <row r="12" spans="1:4" ht="34.200000000000003" thickBot="1">
-      <c r="A12" s="37"/>
-      <c r="B12" s="31"/>
+      <c r="A12" s="32"/>
+      <c r="B12" s="35"/>
       <c r="C12" s="12" t="s">
         <v>55</v>
       </c>
@@ -2058,125 +2058,122 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="16.8">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="33" t="s">
         <v>44</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="29" t="s">
+      <c r="D13" s="33" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="16.8">
-      <c r="A14" s="33"/>
-      <c r="B14" s="30"/>
+      <c r="A14" s="37"/>
+      <c r="B14" s="34"/>
       <c r="C14" s="11"/>
-      <c r="D14" s="30"/>
+      <c r="D14" s="34"/>
     </row>
     <row r="15" spans="1:4" ht="16.8">
-      <c r="A15" s="33"/>
-      <c r="B15" s="30"/>
+      <c r="A15" s="37"/>
+      <c r="B15" s="34"/>
       <c r="C15" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="30"/>
+      <c r="D15" s="34"/>
     </row>
     <row r="16" spans="1:4" ht="16.8">
-      <c r="A16" s="33"/>
-      <c r="B16" s="30"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="34"/>
       <c r="C16" s="11"/>
-      <c r="D16" s="30"/>
+      <c r="D16" s="34"/>
     </row>
     <row r="17" spans="1:4" ht="34.200000000000003" thickBot="1">
-      <c r="A17" s="34"/>
-      <c r="B17" s="31"/>
+      <c r="A17" s="38"/>
+      <c r="B17" s="35"/>
       <c r="C17" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="31"/>
+      <c r="D17" s="35"/>
     </row>
     <row r="18" spans="1:4" ht="33.6">
-      <c r="A18" s="32" t="s">
+      <c r="A18" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="33" t="s">
         <v>44</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="29" t="s">
+      <c r="D18" s="33" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="16.8">
-      <c r="A19" s="33"/>
-      <c r="B19" s="30"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="34"/>
       <c r="C19" s="11"/>
-      <c r="D19" s="30"/>
+      <c r="D19" s="34"/>
     </row>
     <row r="20" spans="1:4" ht="34.200000000000003" thickBot="1">
-      <c r="A20" s="34"/>
-      <c r="B20" s="31"/>
+      <c r="A20" s="38"/>
+      <c r="B20" s="35"/>
       <c r="C20" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="31"/>
+      <c r="D20" s="35"/>
     </row>
     <row r="21" spans="1:4" ht="16.8">
-      <c r="A21" s="32" t="s">
+      <c r="A21" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="33" t="s">
         <v>44</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="29" t="s">
+      <c r="D21" s="33" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="16.8">
-      <c r="A22" s="33"/>
-      <c r="B22" s="30"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="34"/>
       <c r="C22" s="11"/>
-      <c r="D22" s="30"/>
+      <c r="D22" s="34"/>
     </row>
     <row r="23" spans="1:4" ht="16.8">
-      <c r="A23" s="33"/>
-      <c r="B23" s="30"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="34"/>
       <c r="C23" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D23" s="30"/>
+      <c r="D23" s="34"/>
     </row>
     <row r="24" spans="1:4" ht="16.8">
-      <c r="A24" s="33"/>
-      <c r="B24" s="30"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="34"/>
       <c r="C24" s="11"/>
-      <c r="D24" s="30"/>
+      <c r="D24" s="34"/>
     </row>
     <row r="25" spans="1:4" ht="17.399999999999999" thickBot="1">
-      <c r="A25" s="34"/>
-      <c r="B25" s="31"/>
+      <c r="A25" s="38"/>
+      <c r="B25" s="35"/>
       <c r="C25" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="D25" s="31"/>
+      <c r="D25" s="35"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="16">
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B10:B12"/>
     <mergeCell ref="A21:A25"/>
     <mergeCell ref="B21:B25"/>
     <mergeCell ref="D21:D25"/>
@@ -2186,8 +2183,11 @@
     <mergeCell ref="A18:A20"/>
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="D18:D20"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="D7:D9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>